<commit_message>
added exp3 and a little bit of tidying
</commit_message>
<xml_diff>
--- a/manuscript/table_fomatting.xlsx
+++ b/manuscript/table_fomatting.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Documents\Christine\Arbeit\06_Forschungsprojekte\2025_Simultaneous_Adaptation\manuscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246B2BC0-6CF4-4896-8159-42A483F4B7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4861CDC-B061-4A28-9486-BC893475DF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="15" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exp1" sheetId="1" r:id="rId1"/>
     <sheet name="Exp2" sheetId="2" r:id="rId2"/>
+    <sheet name="Exp3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="68">
   <si>
     <t>Chi2</t>
   </si>
@@ -196,6 +197,51 @@
   </si>
   <si>
     <t>tML x SpID: M4 x AdaptCond: 4</t>
+  </si>
+  <si>
+    <t>&lt;.001</t>
+  </si>
+  <si>
+    <t>Pseudoword (PW)</t>
+  </si>
+  <si>
+    <t>tML x PW</t>
+  </si>
+  <si>
+    <t>AdaptCond x PW</t>
+  </si>
+  <si>
+    <t>tML x PW x AdaptCond</t>
+  </si>
+  <si>
+    <t>Model Exp 3</t>
+  </si>
+  <si>
+    <t>tML x AdaptCon</t>
+  </si>
+  <si>
+    <t>PW: PW2*</t>
+  </si>
+  <si>
+    <t>PW: PW3</t>
+  </si>
+  <si>
+    <t>PW: PW4</t>
+  </si>
+  <si>
+    <t>AdaptCond: 2**</t>
+  </si>
+  <si>
+    <t>tML x PW: W3</t>
+  </si>
+  <si>
+    <t>tML x PW: W4</t>
+  </si>
+  <si>
+    <t>tML * Pseudoword * AdaptCond + (1|SpID) + (1 | Participant)</t>
+  </si>
+  <si>
+    <t>tML x PW: W4 x AdaptCond: 2</t>
   </si>
 </sst>
 </file>
@@ -341,7 +387,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -416,6 +462,16 @@
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -722,32 +778,32 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -1112,32 +1168,32 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -1474,32 +1530,32 @@
       <c r="I16" s="12"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
@@ -1847,4 +1903,414 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471F7E79-64BB-4DE4-AA05-18032E94BFE1}">
+  <dimension ref="A2:R19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" style="25" customWidth="1"/>
+    <col min="4" max="4" width="1.28515625" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" customWidth="1"/>
+    <col min="7" max="7" width="4.42578125" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
+    <col min="14" max="14" width="29.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="33">
+        <v>4111.7</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>0.32</v>
+      </c>
+      <c r="G5">
+        <v>0.31559999999999999</v>
+      </c>
+      <c r="H5" s="27">
+        <v>1.012</v>
+      </c>
+      <c r="I5" s="35">
+        <v>0.31141000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="33">
+        <v>452.31</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6">
+        <v>1.65</v>
+      </c>
+      <c r="G6">
+        <v>9.0959999999999999E-2</v>
+      </c>
+      <c r="H6">
+        <v>18.145</v>
+      </c>
+      <c r="I6" s="36" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="33">
+        <v>6.52</v>
+      </c>
+      <c r="C7" s="33">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7">
+        <v>-1.64</v>
+      </c>
+      <c r="G7">
+        <v>0.11907</v>
+      </c>
+      <c r="H7">
+        <v>-13.747</v>
+      </c>
+      <c r="I7" s="36" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="33">
+        <v>40.61</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8">
+        <v>-1.05</v>
+      </c>
+      <c r="G8">
+        <v>0.11574</v>
+      </c>
+      <c r="H8" s="27">
+        <v>-9.0310000000000006</v>
+      </c>
+      <c r="I8" s="36" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9">
+        <v>0.73</v>
+      </c>
+      <c r="C9">
+        <v>0.375</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9">
+        <v>-0.41</v>
+      </c>
+      <c r="G9">
+        <v>0.11477999999999999</v>
+      </c>
+      <c r="H9" s="27">
+        <v>-3.5529999999999999</v>
+      </c>
+      <c r="I9" s="36" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10">
+        <v>0.73</v>
+      </c>
+      <c r="C10">
+        <v>0.86599999999999999</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10">
+        <v>-0.23</v>
+      </c>
+      <c r="G10">
+        <v>0.10882</v>
+      </c>
+      <c r="H10" s="27">
+        <v>-2.133</v>
+      </c>
+      <c r="I10" s="33">
+        <v>3.2960000000000003E-2</v>
+      </c>
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="33">
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="C11" s="33">
+        <v>2.3E-2</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11">
+        <v>0.41</v>
+      </c>
+      <c r="G11">
+        <v>0.13974</v>
+      </c>
+      <c r="H11" s="27">
+        <v>2.9239999999999999</v>
+      </c>
+      <c r="I11" s="33">
+        <v>3.4529999999999999E-3</v>
+      </c>
+      <c r="R11" s="1"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F12">
+        <v>0.68</v>
+      </c>
+      <c r="G12">
+        <v>0.14718000000000001</v>
+      </c>
+      <c r="H12" s="27">
+        <v>4.6289999999999996</v>
+      </c>
+      <c r="I12" s="36" t="s">
+        <v>6</v>
+      </c>
+      <c r="R12" s="1"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="33"/>
+      <c r="C13" s="34"/>
+      <c r="E13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13">
+        <v>-0.56999999999999995</v>
+      </c>
+      <c r="G13">
+        <v>0.19993</v>
+      </c>
+      <c r="H13" s="27">
+        <v>-2.835</v>
+      </c>
+      <c r="I13" s="33">
+        <v>4.5830000000000003E-3</v>
+      </c>
+      <c r="R13" s="1"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R14" s="1"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" s="18"/>
+      <c r="I15" s="19"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="11">
+        <v>7932.7</v>
+      </c>
+      <c r="C16" s="32">
+        <v>8061.3</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="14">
+        <v>0.41839999999999999</v>
+      </c>
+      <c r="G16" s="14">
+        <v>0.64690000000000003</v>
+      </c>
+      <c r="H16" s="14"/>
+      <c r="I16" s="20"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="11">
+        <v>9371</v>
+      </c>
+      <c r="C17" s="22"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0.3352</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0.57899999999999996</v>
+      </c>
+      <c r="H17" s="14"/>
+      <c r="I17" s="20"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6">
+        <v>42</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="6"/>
+      <c r="R18" s="1"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="12">
+        <v>4</v>
+      </c>
+      <c r="C19" s="24"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="B3:I3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
erste vollständige Version an Manuuu
</commit_message>
<xml_diff>
--- a/manuscript/table_fomatting.xlsx
+++ b/manuscript/table_fomatting.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Documents\Christine\Arbeit\06_Forschungsprojekte\2025_Simultaneous_Adaptation\manuscript\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4861CDC-B061-4A28-9486-BC893475DF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9895B2D2-7CB0-4CA8-BE77-9198AB0C3622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exp1" sheetId="1" r:id="rId1"/>
     <sheet name="Exp2" sheetId="2" r:id="rId2"/>
     <sheet name="Exp3" sheetId="3" r:id="rId3"/>
+    <sheet name="Acoustics_Supplemental" sheetId="4" r:id="rId4"/>
+    <sheet name="Exp3_Supplemental4" sheetId="6" r:id="rId5"/>
+    <sheet name="Exp3_Supplemental5" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="93">
   <si>
     <t>Chi2</t>
   </si>
@@ -242,16 +245,92 @@
   </si>
   <si>
     <t>tML x PW: W4 x AdaptCond: 2</t>
+  </si>
+  <si>
+    <t>female speakers</t>
+  </si>
+  <si>
+    <t>male speakers</t>
+  </si>
+  <si>
+    <t>ang</t>
+  </si>
+  <si>
+    <t>fea</t>
+  </si>
+  <si>
+    <t>F0 Mean</t>
+  </si>
+  <si>
+    <t>F0 SD</t>
+  </si>
+  <si>
+    <t>F0 Intonation</t>
+  </si>
+  <si>
+    <t>F0 Glide</t>
+  </si>
+  <si>
+    <t>Alpha Ratio</t>
+  </si>
+  <si>
+    <t>HNR</t>
+  </si>
+  <si>
+    <t>Jitter</t>
+  </si>
+  <si>
+    <t>Shimmer</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>SpSex</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Model Exp 3 - female stimuli only</t>
+  </si>
+  <si>
+    <t>Model Exp 3 - male stimuli only</t>
+  </si>
+  <si>
+    <t>&lt;0.01</t>
+  </si>
+  <si>
+    <t>tML x PW: W2</t>
+  </si>
+  <si>
+    <t>PW: W2 x AdaptCond: 2</t>
+  </si>
+  <si>
+    <t>PW: W3 x AdaptCond: 2</t>
+  </si>
+  <si>
+    <t>PW: W4 x AdaptCond: 2</t>
+  </si>
+  <si>
+    <t>tML x PW: W2 x AdaptCond: 2</t>
+  </si>
+  <si>
+    <t>tML x PW: W3 x AdaptCond: 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -315,15 +394,41 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -346,7 +451,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -383,11 +488,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -455,9 +589,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -473,6 +604,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -481,6 +613,82 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -763,21 +971,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:P17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="25" customWidth="1"/>
-    <col min="4" max="4" width="1.28515625" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="1.33203125" customWidth="1"/>
     <col min="5" max="5" width="27" customWidth="1"/>
     <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="5.42578125" customWidth="1"/>
-    <col min="8" max="8" width="5.85546875" customWidth="1"/>
-    <col min="9" max="9" width="5.28515625" customWidth="1"/>
-    <col min="11" max="11" width="30.42578125" customWidth="1"/>
+    <col min="7" max="7" width="5.44140625" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" customWidth="1"/>
+    <col min="9" max="9" width="5.33203125" customWidth="1"/>
+    <col min="11" max="11" width="30.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="37" t="s">
         <v>25</v>
       </c>
@@ -790,7 +998,7 @@
       <c r="H2" s="38"/>
       <c r="I2" s="38"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -805,7 +1013,7 @@
       <c r="H3" s="39"/>
       <c r="I3" s="39"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -833,8 +1041,8 @@
       </c>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="30" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="7">
@@ -844,7 +1052,7 @@
         <v>6</v>
       </c>
       <c r="D5" s="6"/>
-      <c r="E5" s="31" t="s">
+      <c r="E5" s="30" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="14">
@@ -860,8 +1068,8 @@
         <v>5.1330000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" s="30" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="6">
@@ -871,7 +1079,7 @@
         <v>0.85599999999999998</v>
       </c>
       <c r="D6" s="6"/>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="30" t="s">
         <v>21</v>
       </c>
       <c r="F6" s="14">
@@ -888,8 +1096,8 @@
       </c>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="30" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="6">
@@ -899,7 +1107,7 @@
         <v>0.53600000000000003</v>
       </c>
       <c r="D7" s="6"/>
-      <c r="E7" s="31" t="s">
+      <c r="E7" s="30" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="14">
@@ -916,8 +1124,8 @@
       </c>
       <c r="P7" s="1"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="30" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="7">
@@ -927,7 +1135,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="D8" s="6"/>
-      <c r="E8" s="31" t="s">
+      <c r="E8" s="30" t="s">
         <v>36</v>
       </c>
       <c r="F8" s="14">
@@ -943,8 +1151,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="31" t="s">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="30" t="s">
         <v>31</v>
       </c>
       <c r="B9" s="6">
@@ -954,7 +1162,7 @@
         <v>0.19</v>
       </c>
       <c r="D9" s="6"/>
-      <c r="E9" s="31" t="s">
+      <c r="E9" s="30" t="s">
         <v>23</v>
       </c>
       <c r="F9" s="14">
@@ -970,8 +1178,8 @@
         <v>3.0300000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10" s="30" t="s">
         <v>40</v>
       </c>
       <c r="B10" s="7">
@@ -981,7 +1189,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="30" t="s">
         <v>37</v>
       </c>
       <c r="F10" s="14">
@@ -997,8 +1205,8 @@
         <v>0.97231000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="31" t="s">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11" s="30" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="6">
@@ -1008,7 +1216,7 @@
         <v>0.20699999999999999</v>
       </c>
       <c r="D11" s="6"/>
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="30" t="s">
         <v>38</v>
       </c>
       <c r="F11" s="14">
@@ -1025,12 +1233,12 @@
       </c>
       <c r="P11" s="1"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="22"/>
       <c r="D12" s="6"/>
-      <c r="E12" s="31" t="s">
+      <c r="E12" s="30" t="s">
         <v>39</v>
       </c>
       <c r="F12" s="14">
@@ -1047,7 +1255,7 @@
       </c>
       <c r="P12" s="1"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1066,7 +1274,7 @@
       <c r="H13" s="18"/>
       <c r="I13" s="19"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
@@ -1089,7 +1297,7 @@
       <c r="H14" s="14"/>
       <c r="I14" s="20"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
@@ -1110,7 +1318,7 @@
       <c r="H15" s="14"/>
       <c r="I15" s="20"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>13</v>
       </c>
@@ -1125,7 +1333,7 @@
       <c r="H16" s="10"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>43</v>
       </c>
@@ -1153,21 +1361,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1D741DE-D247-4C24-A11A-47402E21E4AD}">
   <dimension ref="A2:S31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="25" customWidth="1"/>
-    <col min="4" max="4" width="1.28515625" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="1.33203125" customWidth="1"/>
     <col min="5" max="5" width="27" customWidth="1"/>
     <col min="6" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="5.42578125" customWidth="1"/>
-    <col min="8" max="8" width="5.85546875" customWidth="1"/>
+    <col min="7" max="7" width="5.44140625" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" customWidth="1"/>
     <col min="9" max="9" width="6" customWidth="1"/>
-    <col min="14" max="14" width="29.42578125" customWidth="1"/>
+    <col min="14" max="14" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="37" t="s">
         <v>26</v>
       </c>
@@ -1180,7 +1388,7 @@
       <c r="H2" s="38"/>
       <c r="I2" s="38"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -1195,7 +1403,7 @@
       <c r="H3" s="39"/>
       <c r="I3" s="39"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -1222,12 +1430,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="28">
-        <v>1778.33</v>
+        <v>1785.96</v>
       </c>
       <c r="C5" s="21" t="s">
         <v>6</v>
@@ -1237,27 +1445,27 @@
         <v>3</v>
       </c>
       <c r="F5" s="27">
-        <v>-0.18645900000000001</v>
+        <v>-0.16736529999999999</v>
       </c>
       <c r="G5" s="27">
-        <v>0.12334100000000001</v>
+        <v>0.1249952</v>
       </c>
       <c r="H5" s="27">
-        <v>-1.512</v>
-      </c>
-      <c r="I5" s="15">
-        <v>0.13100000000000001</v>
+        <v>-1.339</v>
+      </c>
+      <c r="I5" s="36">
+        <v>0.18057899999999999</v>
       </c>
       <c r="O5" s="27"/>
       <c r="P5" s="27"/>
       <c r="Q5" s="27"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B6" s="28">
-        <v>42.09</v>
+        <v>44</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>6</v>
@@ -1266,14 +1474,14 @@
       <c r="E6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="27">
-        <v>1.7216549999999999</v>
-      </c>
-      <c r="G6" s="27">
-        <v>9.4289999999999999E-2</v>
-      </c>
-      <c r="H6" s="27">
-        <v>18.259</v>
+      <c r="F6" s="28">
+        <v>1.7435683</v>
+      </c>
+      <c r="G6" s="28">
+        <v>9.5468800000000006E-2</v>
+      </c>
+      <c r="H6" s="28">
+        <v>18.263000000000002</v>
       </c>
       <c r="I6" s="16" t="s">
         <v>6</v>
@@ -1283,28 +1491,28 @@
       <c r="Q6" s="27"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="28">
-        <v>6.94</v>
+      <c r="B7" s="32">
+        <v>7.16</v>
       </c>
       <c r="C7" s="21">
-        <v>8.0000000000000002E-3</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="27">
-        <v>-0.30108099999999999</v>
-      </c>
-      <c r="G7" s="27">
-        <v>0.104462</v>
-      </c>
-      <c r="H7" s="27">
-        <v>-2.8820000000000001</v>
+      <c r="F7" s="28">
+        <v>-0.30304170000000002</v>
+      </c>
+      <c r="G7" s="28">
+        <v>0.1049771</v>
+      </c>
+      <c r="H7" s="28">
+        <v>-2.887</v>
       </c>
       <c r="I7" s="17">
         <v>4.0000000000000001E-3</v>
@@ -1313,12 +1521,12 @@
       <c r="P7" s="27"/>
       <c r="Q7" s="27"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="28">
-        <v>31.69</v>
+      <c r="B8" s="32">
+        <v>34.14</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>6</v>
@@ -1328,43 +1536,43 @@
         <v>36</v>
       </c>
       <c r="F8" s="27">
-        <v>-6.5250000000000004E-3</v>
+        <v>7.9049999999999997E-4</v>
       </c>
       <c r="G8" s="27">
-        <v>0.110554</v>
+        <v>0.1114026</v>
       </c>
       <c r="H8" s="27">
-        <v>-5.8999999999999997E-2</v>
-      </c>
-      <c r="I8" s="30">
-        <v>0.95299999999999996</v>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="I8" s="36">
+        <v>0.99433899999999997</v>
       </c>
       <c r="O8" s="27"/>
       <c r="P8" s="27"/>
       <c r="Q8" s="27"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="28">
-        <v>5.82</v>
+      <c r="B9" s="32">
+        <v>5.95</v>
       </c>
       <c r="C9" s="29">
-        <v>1.6E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="27">
-        <v>-0.45649400000000001</v>
-      </c>
-      <c r="G9" s="27">
-        <v>0.12246600000000001</v>
-      </c>
-      <c r="H9" s="27">
-        <v>-3.7280000000000002</v>
+      <c r="F9" s="28">
+        <v>-0.47611969999999998</v>
+      </c>
+      <c r="G9" s="28">
+        <v>0.12354130000000001</v>
+      </c>
+      <c r="H9" s="28">
+        <v>-3.8540000000000001</v>
       </c>
       <c r="I9" s="16" t="s">
         <v>6</v>
@@ -1373,67 +1581,68 @@
       <c r="P9" s="27"/>
       <c r="Q9" s="27"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="28">
-        <v>6.49</v>
+      <c r="B10" s="32">
+        <v>7.21</v>
       </c>
       <c r="C10" s="21">
-        <v>1.0999999999999999E-2</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="27">
-        <v>0.27460299999999999</v>
-      </c>
-      <c r="G10" s="27">
-        <v>0.139819</v>
-      </c>
-      <c r="H10" s="27">
-        <v>1.964</v>
+      <c r="F10" s="28">
+        <v>0.28286519999999998</v>
+      </c>
+      <c r="G10" s="28">
+        <v>0.1416886</v>
+      </c>
+      <c r="H10" s="28">
+        <v>1.996</v>
       </c>
       <c r="I10" s="17">
-        <v>4.9000000000000002E-2</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="O10" s="27"/>
       <c r="P10" s="27"/>
       <c r="Q10" s="27"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="27">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="C11" s="22">
-        <v>0.55200000000000005</v>
+        <v>0.52800000000000002</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="27">
-        <v>-0.39059199999999999</v>
-      </c>
-      <c r="G11" s="27">
-        <v>0.153449</v>
-      </c>
-      <c r="H11" s="27">
-        <v>-2.5449999999999999</v>
+      <c r="F11" s="28">
+        <v>-0.41373349999999998</v>
+      </c>
+      <c r="G11" s="28">
+        <v>0.15421170000000001</v>
+      </c>
+      <c r="H11" s="28">
+        <v>-2.6829999999999998</v>
       </c>
       <c r="I11" s="16">
-        <v>1.0999999999999999E-2</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="O11" s="27"/>
       <c r="P11" s="27"/>
       <c r="Q11" s="27"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="R11" s="36"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="22"/>
@@ -1442,22 +1651,24 @@
         <v>48</v>
       </c>
       <c r="F12" s="27">
-        <v>-0.108917</v>
+        <v>-0.1166325</v>
       </c>
       <c r="G12" s="27">
-        <v>0.183084</v>
+        <v>0.18469379999999999</v>
       </c>
       <c r="H12" s="27">
-        <v>-0.59499999999999997</v>
-      </c>
-      <c r="I12" s="15">
-        <v>0.55200000000000005</v>
+        <v>-0.63100000000000001</v>
+      </c>
+      <c r="I12" s="36">
+        <v>0.52771900000000005</v>
       </c>
       <c r="O12" s="27"/>
       <c r="P12" s="27"/>
       <c r="Q12" s="27"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="R12" s="36"/>
+      <c r="S12" s="1"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
@@ -1475,36 +1686,46 @@
       </c>
       <c r="H13" s="18"/>
       <c r="I13" s="19"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27"/>
+      <c r="R13" s="36"/>
+      <c r="S13" s="1"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="11">
-        <v>4503.1000000000004</v>
-      </c>
-      <c r="C14" s="32">
-        <v>4561.2</v>
+        <v>4460</v>
+      </c>
+      <c r="C14" s="31">
+        <v>4518</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="14">
-        <v>0.39560000000000001</v>
+        <v>0.41</v>
       </c>
       <c r="G14" s="14">
-        <v>0.629</v>
+        <v>0.64</v>
       </c>
       <c r="H14" s="14"/>
       <c r="I14" s="20"/>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O14" s="27"/>
+      <c r="P14" s="27"/>
+      <c r="Q14" s="27"/>
+      <c r="R14" s="36"/>
+      <c r="S14" s="1"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="11">
-        <v>4704</v>
+        <v>4677</v>
       </c>
       <c r="C15" s="22"/>
       <c r="D15" s="6"/>
@@ -1513,8 +1734,12 @@
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
       <c r="I15" s="20"/>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
+      <c r="R15" s="36"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
         <v>13</v>
       </c>
@@ -1528,8 +1753,12 @@
       <c r="G16" s="12"/>
       <c r="H16" s="13"/>
       <c r="I16" s="12"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O16" s="27"/>
+      <c r="P16" s="27"/>
+      <c r="Q16" s="27"/>
+      <c r="R16" s="36"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" s="37" t="s">
         <v>44</v>
       </c>
@@ -1541,8 +1770,12 @@
       <c r="G17" s="38"/>
       <c r="H17" s="38"/>
       <c r="I17" s="38"/>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O17" s="27"/>
+      <c r="P17" s="27"/>
+      <c r="Q17" s="27"/>
+      <c r="R17" s="36"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1556,8 +1789,12 @@
       <c r="G18" s="39"/>
       <c r="H18" s="39"/>
       <c r="I18" s="39"/>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
+      <c r="Q18" s="27"/>
+      <c r="R18" s="36"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>14</v>
       </c>
@@ -1583,13 +1820,17 @@
       <c r="I19" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="27"/>
+      <c r="R19" s="36"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="27">
-        <v>1846.07</v>
+      <c r="B20" s="28">
+        <v>1860.19</v>
       </c>
       <c r="C20" s="21" t="s">
         <v>6</v>
@@ -1598,14 +1839,14 @@
       <c r="E20" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F20" s="27">
-        <v>-1.37954</v>
-      </c>
-      <c r="G20" s="27">
-        <v>0.15271999999999999</v>
-      </c>
-      <c r="H20" s="27">
-        <v>-9.0329999999999995</v>
+      <c r="F20" s="28">
+        <v>-1.3763799999999999</v>
+      </c>
+      <c r="G20" s="28">
+        <v>0.15393999999999999</v>
+      </c>
+      <c r="H20" s="28">
+        <v>-8.9410000000000007</v>
       </c>
       <c r="I20" s="16" t="s">
         <v>6</v>
@@ -1615,12 +1856,12 @@
       <c r="Q20" s="27"/>
       <c r="S20" s="1"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="27">
-        <v>433.77</v>
+      <c r="B21" s="28">
+        <v>441.93</v>
       </c>
       <c r="C21" s="21" t="s">
         <v>6</v>
@@ -1629,14 +1870,14 @@
       <c r="E21" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="27">
-        <v>1.49458</v>
-      </c>
-      <c r="G21" s="27">
-        <v>9.6570000000000003E-2</v>
-      </c>
-      <c r="H21" s="27">
-        <v>15.477</v>
+      <c r="F21" s="28">
+        <v>1.4970699999999999</v>
+      </c>
+      <c r="G21" s="28">
+        <v>9.6759999999999999E-2</v>
+      </c>
+      <c r="H21" s="28">
+        <v>15.473000000000001</v>
       </c>
       <c r="I21" s="16" t="s">
         <v>6</v>
@@ -1646,12 +1887,12 @@
       <c r="Q21" s="27"/>
       <c r="S21" s="1"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="27">
-        <v>36.31</v>
+      <c r="B22" s="28">
+        <v>34.590000000000003</v>
       </c>
       <c r="C22" s="21" t="s">
         <v>6</v>
@@ -1660,14 +1901,14 @@
       <c r="E22" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F22" s="27">
-        <v>1.8655999999999999</v>
-      </c>
-      <c r="G22" s="27">
-        <v>0.12761</v>
-      </c>
-      <c r="H22" s="27">
-        <v>14.62</v>
+      <c r="F22" s="28">
+        <v>1.8795999999999999</v>
+      </c>
+      <c r="G22" s="28">
+        <v>0.12822</v>
+      </c>
+      <c r="H22" s="28">
+        <v>14.66</v>
       </c>
       <c r="I22" s="16" t="s">
         <v>6</v>
@@ -1677,12 +1918,12 @@
       <c r="Q22" s="27"/>
       <c r="S22" s="1"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="27">
-        <v>54.6</v>
+      <c r="B23" s="28">
+        <v>57.57</v>
       </c>
       <c r="C23" s="21" t="s">
         <v>6</v>
@@ -1691,14 +1932,14 @@
       <c r="E23" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="27">
-        <v>-0.46879999999999999</v>
-      </c>
-      <c r="G23" s="27">
-        <v>0.13547999999999999</v>
-      </c>
-      <c r="H23" s="27">
-        <v>-3.46</v>
+      <c r="F23" s="28">
+        <v>-0.46951999999999999</v>
+      </c>
+      <c r="G23" s="28">
+        <v>0.13558999999999999</v>
+      </c>
+      <c r="H23" s="28">
+        <v>-3.4630000000000001</v>
       </c>
       <c r="I23" s="16" t="s">
         <v>6</v>
@@ -1707,28 +1948,28 @@
       <c r="P23" s="27"/>
       <c r="Q23" s="27"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B24" s="27">
-        <v>2.88</v>
-      </c>
-      <c r="C24" s="8">
-        <v>0.09</v>
+        <v>2.61</v>
+      </c>
+      <c r="C24" s="36">
+        <v>0.106</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F24" s="27">
-        <v>0.89302999999999999</v>
-      </c>
-      <c r="G24" s="27">
-        <v>0.15518000000000001</v>
-      </c>
-      <c r="H24" s="27">
-        <v>5.7549999999999999</v>
+      <c r="F24" s="28">
+        <v>0.91720000000000002</v>
+      </c>
+      <c r="G24" s="28">
+        <v>0.15639</v>
+      </c>
+      <c r="H24" s="28">
+        <v>5.8650000000000002</v>
       </c>
       <c r="I24" s="16" t="s">
         <v>6</v>
@@ -1738,67 +1979,67 @@
       <c r="Q24" s="27"/>
       <c r="R24" s="1"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B25" s="27">
-        <v>0.66</v>
-      </c>
-      <c r="C25" s="22">
-        <v>0.41499999999999998</v>
+        <v>0.48</v>
+      </c>
+      <c r="C25" s="36">
+        <v>0.49</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6" t="s">
         <v>50</v>
       </c>
       <c r="F25" s="27">
-        <v>-7.8939999999999996E-2</v>
+        <v>-7.5069999999999998E-2</v>
       </c>
       <c r="G25" s="27">
-        <v>0.14018</v>
+        <v>0.14052999999999999</v>
       </c>
       <c r="H25" s="27">
-        <v>-0.56299999999999994</v>
-      </c>
-      <c r="I25" s="15">
-        <v>0.57299999999999995</v>
+        <v>-0.53400000000000003</v>
+      </c>
+      <c r="I25" s="36">
+        <v>0.59323499999999996</v>
       </c>
       <c r="O25" s="27"/>
       <c r="P25" s="27"/>
       <c r="Q25" s="27"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B26" s="27">
-        <v>0.93</v>
-      </c>
-      <c r="C26" s="22">
-        <v>0.33600000000000002</v>
+        <v>0.85</v>
+      </c>
+      <c r="C26">
+        <v>0.35699999999999998</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
         <v>51</v>
       </c>
       <c r="F26" s="27">
-        <v>-0.14815</v>
+        <v>-0.12609999999999999</v>
       </c>
       <c r="G26" s="27">
-        <v>0.18148</v>
+        <v>0.18235000000000001</v>
       </c>
       <c r="H26" s="27">
-        <v>-0.81599999999999995</v>
-      </c>
-      <c r="I26" s="30">
-        <v>0.41399999999999998</v>
+        <v>-0.69099999999999995</v>
+      </c>
+      <c r="I26" s="36">
+        <v>0.48925800000000003</v>
       </c>
       <c r="O26" s="27"/>
       <c r="P26" s="27"/>
       <c r="Q26" s="27"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" s="6"/>
       <c r="B27" s="27"/>
       <c r="C27" s="22"/>
@@ -1807,22 +2048,22 @@
         <v>52</v>
       </c>
       <c r="F27" s="27">
-        <v>-0.20594000000000001</v>
+        <v>-0.19878999999999999</v>
       </c>
       <c r="G27" s="27">
-        <v>0.21435000000000001</v>
+        <v>0.21618999999999999</v>
       </c>
       <c r="H27" s="27">
-        <v>-0.96099999999999997</v>
-      </c>
-      <c r="I27" s="15">
-        <v>0.33700000000000002</v>
+        <v>-0.91900000000000004</v>
+      </c>
+      <c r="I27" s="36">
+        <v>0.35784100000000002</v>
       </c>
       <c r="O27" s="27"/>
       <c r="P27" s="27"/>
       <c r="Q27" s="27"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>11</v>
       </c>
@@ -1841,35 +2082,35 @@
       <c r="H28" s="18"/>
       <c r="I28" s="19"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B29" s="11">
-        <v>3855.1</v>
-      </c>
-      <c r="C29" s="32">
-        <v>3913.2</v>
+        <v>3816</v>
+      </c>
+      <c r="C29" s="31">
+        <v>3874</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
         <v>8</v>
       </c>
       <c r="F29" s="14">
-        <v>0.63349999999999995</v>
+        <v>0.65</v>
       </c>
       <c r="G29" s="14">
-        <v>0.79590000000000005</v>
+        <v>0.81</v>
       </c>
       <c r="H29" s="14"/>
       <c r="I29" s="20"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B30" s="11">
-        <v>4704</v>
+        <v>4682</v>
       </c>
       <c r="C30" s="22"/>
       <c r="D30" s="6"/>
@@ -1879,7 +2120,7 @@
       <c r="H30" s="14"/>
       <c r="I30" s="20"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
         <v>13</v>
       </c>
@@ -1908,22 +2149,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471F7E79-64BB-4DE4-AA05-18032E94BFE1}">
   <dimension ref="A2:R19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="25" customWidth="1"/>
-    <col min="4" max="4" width="1.28515625" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" customWidth="1"/>
-    <col min="8" max="8" width="6.42578125" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="1.33203125" customWidth="1"/>
+    <col min="5" max="5" width="24.5546875" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" customWidth="1"/>
+    <col min="7" max="7" width="4.44140625" customWidth="1"/>
+    <col min="8" max="8" width="6.44140625" customWidth="1"/>
     <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="14" max="14" width="29.7109375" customWidth="1"/>
-    <col min="15" max="15" width="22.42578125" customWidth="1"/>
+    <col min="14" max="14" width="29.6640625" customWidth="1"/>
+    <col min="15" max="15" width="22.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="37" t="s">
         <v>58</v>
       </c>
@@ -1936,7 +2177,7 @@
       <c r="H2" s="38"/>
       <c r="I2" s="38"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -1951,7 +2192,7 @@
       <c r="H3" s="39"/>
       <c r="I3" s="39"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -1978,14 +2219,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="33">
+      <c r="B5" s="32">
         <v>4111.7</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="33" t="s">
         <v>53</v>
       </c>
       <c r="D5" s="6"/>
@@ -2001,18 +2242,18 @@
       <c r="H5" s="27">
         <v>1.012</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I5" s="34">
         <v>0.31141000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="32">
         <v>452.31</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="33" t="s">
         <v>53</v>
       </c>
       <c r="D6" s="6"/>
@@ -2028,18 +2269,18 @@
       <c r="H6">
         <v>18.145</v>
       </c>
-      <c r="I6" s="36" t="s">
+      <c r="I6" s="35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="33">
+      <c r="B7" s="32">
         <v>6.52</v>
       </c>
-      <c r="C7" s="33">
+      <c r="C7" s="32">
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="D7" s="6"/>
@@ -2055,18 +2296,18 @@
       <c r="H7">
         <v>-13.747</v>
       </c>
-      <c r="I7" s="36" t="s">
+      <c r="I7" s="35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="33">
+      <c r="B8" s="32">
         <v>40.61</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="33" t="s">
         <v>53</v>
       </c>
       <c r="D8" s="6"/>
@@ -2082,11 +2323,11 @@
       <c r="H8" s="27">
         <v>-9.0310000000000006</v>
       </c>
-      <c r="I8" s="36" t="s">
+      <c r="I8" s="35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>59</v>
       </c>
@@ -2109,11 +2350,11 @@
       <c r="H9" s="27">
         <v>-3.5529999999999999</v>
       </c>
-      <c r="I9" s="36" t="s">
+      <c r="I9" s="35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>56</v>
       </c>
@@ -2136,19 +2377,19 @@
       <c r="H10" s="27">
         <v>-2.133</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="32">
         <v>3.2960000000000003E-2</v>
       </c>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="33">
+      <c r="B11" s="32">
         <v>9.5399999999999991</v>
       </c>
-      <c r="C11" s="33">
+      <c r="C11" s="32">
         <v>2.3E-2</v>
       </c>
       <c r="D11" s="6"/>
@@ -2164,12 +2405,12 @@
       <c r="H11" s="27">
         <v>2.9239999999999999</v>
       </c>
-      <c r="I11" s="33">
+      <c r="I11" s="32">
         <v>3.4529999999999999E-3</v>
       </c>
       <c r="R11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
         <v>65</v>
@@ -2183,15 +2424,15 @@
       <c r="H12" s="27">
         <v>4.6289999999999996</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="I12" s="35" t="s">
         <v>6</v>
       </c>
       <c r="R12" s="1"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="34"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="33"/>
       <c r="E13" s="6" t="s">
         <v>67</v>
       </c>
@@ -2204,15 +2445,15 @@
       <c r="H13" s="27">
         <v>-2.835</v>
       </c>
-      <c r="I13" s="33">
+      <c r="I13" s="32">
         <v>4.5830000000000003E-3</v>
       </c>
       <c r="R13" s="1"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="R14" s="1"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
@@ -2231,14 +2472,14 @@
       <c r="H15" s="18"/>
       <c r="I15" s="19"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="11">
         <v>7932.7</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="31">
         <v>8061.3</v>
       </c>
       <c r="D16" s="6"/>
@@ -2254,7 +2495,7 @@
       <c r="H16" s="14"/>
       <c r="I16" s="20"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>12</v>
       </c>
@@ -2275,7 +2516,7 @@
       <c r="H17" s="14"/>
       <c r="I17" s="20"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>13</v>
       </c>
@@ -2291,7 +2532,7 @@
       <c r="I18" s="6"/>
       <c r="R18" s="1"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>43</v>
       </c>
@@ -2313,4 +2554,1902 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081E287B-9939-4347-A502-BE07CB24DC4F}">
+  <dimension ref="A1:Q47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="7.5546875" customWidth="1"/>
+    <col min="7" max="7" width="5.33203125" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" customWidth="1"/>
+    <col min="9" max="9" width="7.77734375" customWidth="1"/>
+    <col min="10" max="10" width="10.77734375" customWidth="1"/>
+    <col min="11" max="11" width="8.44140625" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="40"/>
+      <c r="B1" s="49" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49" t="s">
+        <v>69</v>
+      </c>
+      <c r="E1" s="49"/>
+    </row>
+    <row r="2" spans="1:17" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="42"/>
+      <c r="B2" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="44" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="45" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="41">
+        <v>366</v>
+      </c>
+      <c r="C3" s="41">
+        <v>288</v>
+      </c>
+      <c r="D3" s="41">
+        <v>264</v>
+      </c>
+      <c r="E3" s="41">
+        <v>205</v>
+      </c>
+      <c r="K3" s="51"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="51"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="50"/>
+      <c r="Q3" s="36"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="46" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="52">
+        <v>67.128749999999997</v>
+      </c>
+      <c r="C4" s="52">
+        <v>19.03</v>
+      </c>
+      <c r="D4" s="52">
+        <v>45.627499999999998</v>
+      </c>
+      <c r="E4" s="52">
+        <v>26.796250000000001</v>
+      </c>
+      <c r="K4" s="51"/>
+      <c r="L4" s="51"/>
+      <c r="M4" s="51"/>
+      <c r="N4" s="51"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="50"/>
+      <c r="Q4" s="36"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="41">
+        <v>259</v>
+      </c>
+      <c r="C5" s="41">
+        <v>79</v>
+      </c>
+      <c r="D5" s="41">
+        <v>171</v>
+      </c>
+      <c r="E5" s="41">
+        <v>95</v>
+      </c>
+      <c r="K5" s="51"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="51"/>
+      <c r="N5" s="51"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="50"/>
+      <c r="Q5" s="36"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="46" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="41">
+        <v>-60</v>
+      </c>
+      <c r="C6" s="41">
+        <v>3</v>
+      </c>
+      <c r="D6" s="41">
+        <v>-41</v>
+      </c>
+      <c r="E6" s="41">
+        <v>12</v>
+      </c>
+      <c r="K6" s="51"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="51"/>
+      <c r="N6" s="51"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="50"/>
+      <c r="Q6" s="36"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="54">
+        <v>1</v>
+      </c>
+      <c r="C7" s="54">
+        <v>2.2875000000000001</v>
+      </c>
+      <c r="D7" s="54">
+        <v>1.075</v>
+      </c>
+      <c r="E7" s="54">
+        <v>2.2749999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="41">
+        <v>12.8</v>
+      </c>
+      <c r="C8" s="41">
+        <v>21.3</v>
+      </c>
+      <c r="D8" s="41">
+        <v>7.3</v>
+      </c>
+      <c r="E8" s="41">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="41">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="C9" s="41">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="D9" s="41">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="E9" s="41">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="46" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="55">
+        <v>3.5467499999999999E-2</v>
+      </c>
+      <c r="C10" s="55">
+        <v>1.3421249999999999E-2</v>
+      </c>
+      <c r="D10" s="55">
+        <v>6.2792500000000001E-2</v>
+      </c>
+      <c r="E10" s="55">
+        <v>1.265375E-2</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="51"/>
+    </row>
+    <row r="11" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="47" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="48">
+        <v>885</v>
+      </c>
+      <c r="C11" s="48">
+        <v>760</v>
+      </c>
+      <c r="D11" s="48">
+        <v>731</v>
+      </c>
+      <c r="E11" s="48">
+        <v>854</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="51"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="I12" s="36"/>
+      <c r="J12" s="51"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="I13" s="36"/>
+      <c r="J13" s="51"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="60" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="61" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" s="61" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="61" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="62">
+        <v>20</v>
+      </c>
+      <c r="C16" s="52">
+        <v>298.23750000000001</v>
+      </c>
+      <c r="D16" s="52">
+        <v>21.171250000000001</v>
+      </c>
+      <c r="E16" s="52">
+        <v>90.0625</v>
+      </c>
+      <c r="F16" s="52">
+        <v>-20.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="62">
+        <v>30</v>
+      </c>
+      <c r="C17" s="52">
+        <v>304.27499999999998</v>
+      </c>
+      <c r="D17" s="52">
+        <v>25.08</v>
+      </c>
+      <c r="E17" s="52">
+        <v>101.58750000000001</v>
+      </c>
+      <c r="F17" s="52">
+        <v>-26.962499999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="62">
+        <v>40</v>
+      </c>
+      <c r="C18" s="52">
+        <v>310.73750000000001</v>
+      </c>
+      <c r="D18" s="52">
+        <v>30.137499999999999</v>
+      </c>
+      <c r="E18" s="52">
+        <v>117.9375</v>
+      </c>
+      <c r="F18" s="52">
+        <v>-34.112499999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="62">
+        <v>50</v>
+      </c>
+      <c r="C19" s="52">
+        <v>317.55</v>
+      </c>
+      <c r="D19" s="52">
+        <v>36.073749999999997</v>
+      </c>
+      <c r="E19" s="52">
+        <v>139.36250000000001</v>
+      </c>
+      <c r="F19" s="52">
+        <v>-40.4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="62">
+        <v>60</v>
+      </c>
+      <c r="C20" s="52">
+        <v>325.22500000000002</v>
+      </c>
+      <c r="D20" s="52">
+        <v>42.19</v>
+      </c>
+      <c r="E20" s="52">
+        <v>165.28749999999999</v>
+      </c>
+      <c r="F20" s="52">
+        <v>-50.487499999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="62">
+        <v>70</v>
+      </c>
+      <c r="C21" s="52">
+        <v>333.58749999999998</v>
+      </c>
+      <c r="D21" s="52">
+        <v>48.628749999999997</v>
+      </c>
+      <c r="E21" s="52">
+        <v>185.98750000000001</v>
+      </c>
+      <c r="F21" s="52">
+        <v>-55.35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="63">
+        <v>80</v>
+      </c>
+      <c r="C22" s="59">
+        <v>343.4</v>
+      </c>
+      <c r="D22" s="59">
+        <v>54.784999999999997</v>
+      </c>
+      <c r="E22" s="59">
+        <v>208.2</v>
+      </c>
+      <c r="F22" s="59">
+        <v>-54.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="62">
+        <v>20</v>
+      </c>
+      <c r="C23" s="52">
+        <v>212.47499999999999</v>
+      </c>
+      <c r="D23" s="52">
+        <v>27.192499999999999</v>
+      </c>
+      <c r="E23" s="52">
+        <v>98.075000000000003</v>
+      </c>
+      <c r="F23" s="52">
+        <v>-8.1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="62">
+        <v>30</v>
+      </c>
+      <c r="C24" s="52">
+        <v>216.47499999999999</v>
+      </c>
+      <c r="D24" s="52">
+        <v>28.62125</v>
+      </c>
+      <c r="E24" s="52">
+        <v>104.27500000000001</v>
+      </c>
+      <c r="F24" s="52">
+        <v>-17.6875</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" s="62">
+        <v>40</v>
+      </c>
+      <c r="C25" s="52">
+        <v>221.23750000000001</v>
+      </c>
+      <c r="D25" s="52">
+        <v>30.353750000000002</v>
+      </c>
+      <c r="E25" s="52">
+        <v>110.175</v>
+      </c>
+      <c r="F25" s="52">
+        <v>-21.462499999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B26" s="62">
+        <v>50</v>
+      </c>
+      <c r="C26" s="52">
+        <v>226.03749999999999</v>
+      </c>
+      <c r="D26" s="52">
+        <v>32.946249999999999</v>
+      </c>
+      <c r="E26" s="52">
+        <v>119.21250000000001</v>
+      </c>
+      <c r="F26" s="52">
+        <v>-28.975000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="62">
+        <v>60</v>
+      </c>
+      <c r="C27" s="52">
+        <v>231.61250000000001</v>
+      </c>
+      <c r="D27" s="52">
+        <v>35.71</v>
+      </c>
+      <c r="E27" s="52">
+        <v>128.44999999999999</v>
+      </c>
+      <c r="F27" s="52">
+        <v>-34.637500000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="62">
+        <v>70</v>
+      </c>
+      <c r="C28" s="52">
+        <v>237.76249999999999</v>
+      </c>
+      <c r="D28" s="52">
+        <v>38.493749999999999</v>
+      </c>
+      <c r="E28" s="52">
+        <v>137.65</v>
+      </c>
+      <c r="F28" s="52">
+        <v>-37.725000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="63" t="s">
+        <v>83</v>
+      </c>
+      <c r="B29" s="63">
+        <v>80</v>
+      </c>
+      <c r="C29" s="59">
+        <v>244.2</v>
+      </c>
+      <c r="D29" s="59">
+        <v>41.895000000000003</v>
+      </c>
+      <c r="E29" s="59">
+        <v>149.96250000000001</v>
+      </c>
+      <c r="F29" s="59">
+        <v>-45.287500000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="60" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" s="60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="61" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="61" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="F33" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="G33" s="61" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="62">
+        <v>20</v>
+      </c>
+      <c r="C34" s="54">
+        <v>1.8625</v>
+      </c>
+      <c r="D34" s="54">
+        <v>20.75</v>
+      </c>
+      <c r="E34" s="55">
+        <v>2.6337499999999998E-3</v>
+      </c>
+      <c r="F34" s="55">
+        <v>9.4774999999999998E-3</v>
+      </c>
+      <c r="G34" s="52">
+        <v>785.4375</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B35" s="62">
+        <v>30</v>
+      </c>
+      <c r="C35" s="54">
+        <v>1.7</v>
+      </c>
+      <c r="D35" s="54">
+        <v>19.8</v>
+      </c>
+      <c r="E35" s="55">
+        <v>2.5937500000000001E-3</v>
+      </c>
+      <c r="F35" s="55">
+        <v>1.0619999999999999E-2</v>
+      </c>
+      <c r="G35" s="52">
+        <v>797.95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" s="62">
+        <v>40</v>
+      </c>
+      <c r="C36" s="54">
+        <v>1.55</v>
+      </c>
+      <c r="D36" s="54">
+        <v>18.774999999999999</v>
+      </c>
+      <c r="E36" s="55">
+        <v>2.7637500000000001E-3</v>
+      </c>
+      <c r="F36" s="55">
+        <v>1.3022499999999999E-2</v>
+      </c>
+      <c r="G36" s="52">
+        <v>811.66250000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B37" s="62">
+        <v>50</v>
+      </c>
+      <c r="C37" s="54">
+        <v>1.4125000000000001</v>
+      </c>
+      <c r="D37" s="54">
+        <v>17.875</v>
+      </c>
+      <c r="E37" s="55">
+        <v>2.65125E-3</v>
+      </c>
+      <c r="F37" s="55">
+        <v>1.650625E-2</v>
+      </c>
+      <c r="G37" s="52">
+        <v>824.75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B38" s="62">
+        <v>60</v>
+      </c>
+      <c r="C38" s="54">
+        <v>1.325</v>
+      </c>
+      <c r="D38" s="54">
+        <v>16.95</v>
+      </c>
+      <c r="E38" s="55">
+        <v>2.6337499999999998E-3</v>
+      </c>
+      <c r="F38" s="55">
+        <v>2.225125E-2</v>
+      </c>
+      <c r="G38" s="52">
+        <v>833.07500000000005</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="62">
+        <v>70</v>
+      </c>
+      <c r="C39" s="54">
+        <v>1.2250000000000001</v>
+      </c>
+      <c r="D39" s="54">
+        <v>16.087499999999999</v>
+      </c>
+      <c r="E39" s="55">
+        <v>2.8487500000000002E-3</v>
+      </c>
+      <c r="F39" s="55">
+        <v>2.3885E-2</v>
+      </c>
+      <c r="G39" s="52">
+        <v>845.21249999999998</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="63" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="63">
+        <v>80</v>
+      </c>
+      <c r="C40" s="57">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="D40" s="57">
+        <v>15.237500000000001</v>
+      </c>
+      <c r="E40" s="58">
+        <v>2.7325000000000001E-3</v>
+      </c>
+      <c r="F40" s="58">
+        <v>2.5950000000000001E-2</v>
+      </c>
+      <c r="G40" s="59">
+        <v>859.58749999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" s="62">
+        <v>20</v>
+      </c>
+      <c r="C41" s="54">
+        <v>1.9</v>
+      </c>
+      <c r="D41" s="54">
+        <v>17.524999999999999</v>
+      </c>
+      <c r="E41" s="55">
+        <v>3.50125E-3</v>
+      </c>
+      <c r="F41" s="55">
+        <v>1.410875E-2</v>
+      </c>
+      <c r="G41" s="52">
+        <v>830.76250000000005</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" s="62">
+        <v>30</v>
+      </c>
+      <c r="C42" s="54">
+        <v>1.7375</v>
+      </c>
+      <c r="D42" s="54">
+        <v>16.112500000000001</v>
+      </c>
+      <c r="E42" s="55">
+        <v>3.9824999999999999E-3</v>
+      </c>
+      <c r="F42" s="55">
+        <v>1.7864999999999999E-2</v>
+      </c>
+      <c r="G42" s="52">
+        <v>816.47500000000002</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B43" s="62">
+        <v>40</v>
+      </c>
+      <c r="C43" s="54">
+        <v>1.575</v>
+      </c>
+      <c r="D43" s="54">
+        <v>14.675000000000001</v>
+      </c>
+      <c r="E43" s="55">
+        <v>4.2224999999999997E-3</v>
+      </c>
+      <c r="F43" s="55">
+        <v>2.3706250000000002E-2</v>
+      </c>
+      <c r="G43" s="52">
+        <v>804.38750000000005</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="62">
+        <v>50</v>
+      </c>
+      <c r="C44" s="54">
+        <v>1.4750000000000001</v>
+      </c>
+      <c r="D44" s="54">
+        <v>13.1625</v>
+      </c>
+      <c r="E44" s="55">
+        <v>4.9512499999999999E-3</v>
+      </c>
+      <c r="F44" s="55">
+        <v>2.9309999999999999E-2</v>
+      </c>
+      <c r="G44" s="52">
+        <v>791.0625</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B45" s="62">
+        <v>60</v>
+      </c>
+      <c r="C45" s="54">
+        <v>1.3625</v>
+      </c>
+      <c r="D45" s="54">
+        <v>11.85</v>
+      </c>
+      <c r="E45" s="55">
+        <v>5.3825000000000001E-3</v>
+      </c>
+      <c r="F45" s="55">
+        <v>3.3579999999999999E-2</v>
+      </c>
+      <c r="G45" s="52">
+        <v>776.48749999999995</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="B46" s="62">
+        <v>70</v>
+      </c>
+      <c r="C46" s="54">
+        <v>1.2749999999999999</v>
+      </c>
+      <c r="D46" s="54">
+        <v>10.6625</v>
+      </c>
+      <c r="E46" s="55">
+        <v>5.5975E-3</v>
+      </c>
+      <c r="F46" s="55">
+        <v>4.1794999999999999E-2</v>
+      </c>
+      <c r="G46" s="52">
+        <v>767.05</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="63" t="s">
+        <v>83</v>
+      </c>
+      <c r="B47" s="63">
+        <v>80</v>
+      </c>
+      <c r="C47" s="57">
+        <v>1.2124999999999999</v>
+      </c>
+      <c r="D47" s="57">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="E47" s="58">
+        <v>6.4087500000000004E-3</v>
+      </c>
+      <c r="F47" s="58">
+        <v>4.473125E-2</v>
+      </c>
+      <c r="G47" s="59">
+        <v>756.22500000000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2956A686-49A1-4B69-AD96-1F2B3DE22FA3}">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="4" max="4" width="8.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="53">
+        <v>0.31946999999999998</v>
+      </c>
+      <c r="C2" s="53">
+        <v>0.31559999999999999</v>
+      </c>
+      <c r="D2" s="53">
+        <v>1.012</v>
+      </c>
+      <c r="E2" s="55">
+        <v>0.31141000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="65">
+        <v>1.6504099999999999</v>
+      </c>
+      <c r="C3" s="65">
+        <v>9.0959999999999999E-2</v>
+      </c>
+      <c r="D3" s="65">
+        <v>18.145</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="65">
+        <v>-1.6368100000000001</v>
+      </c>
+      <c r="C4" s="65">
+        <v>0.11907</v>
+      </c>
+      <c r="D4" s="65">
+        <v>-13.747</v>
+      </c>
+      <c r="E4" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="65">
+        <v>-1.04521</v>
+      </c>
+      <c r="C5" s="65">
+        <v>0.11574</v>
+      </c>
+      <c r="D5" s="65">
+        <v>-9.0310000000000006</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="53">
+        <v>-0.40783000000000003</v>
+      </c>
+      <c r="C6" s="53">
+        <v>0.11477999999999999</v>
+      </c>
+      <c r="D6" s="53">
+        <v>-3.5529999999999999</v>
+      </c>
+      <c r="E6" s="55">
+        <v>3.8099999999999999E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="53">
+        <v>-0.23205999999999999</v>
+      </c>
+      <c r="C7" s="53">
+        <v>0.10882</v>
+      </c>
+      <c r="D7" s="53">
+        <v>-2.133</v>
+      </c>
+      <c r="E7" s="55">
+        <v>3.2960000000000003E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="53">
+        <v>-3.2820000000000002E-2</v>
+      </c>
+      <c r="C8" s="53">
+        <v>0.1328</v>
+      </c>
+      <c r="D8" s="53">
+        <v>-0.247</v>
+      </c>
+      <c r="E8" s="55">
+        <v>0.80476700000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="65">
+        <v>0.40862999999999999</v>
+      </c>
+      <c r="C9" s="65">
+        <v>0.13974</v>
+      </c>
+      <c r="D9" s="65">
+        <v>2.9239999999999999</v>
+      </c>
+      <c r="E9" s="64">
+        <v>3.4529999999999999E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="65">
+        <v>0.68128</v>
+      </c>
+      <c r="C10" s="65">
+        <v>0.14718000000000001</v>
+      </c>
+      <c r="D10" s="65">
+        <v>4.6289999999999996</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="53">
+        <v>0.12286</v>
+      </c>
+      <c r="C11" s="53">
+        <v>0.12966</v>
+      </c>
+      <c r="D11" s="53">
+        <v>0.94799999999999995</v>
+      </c>
+      <c r="E11" s="55">
+        <v>0.34334999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="53">
+        <v>9.647E-2</v>
+      </c>
+      <c r="C12" s="53">
+        <v>0.16916999999999999</v>
+      </c>
+      <c r="D12" s="53">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="E12" s="55">
+        <v>0.56849300000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="53">
+        <v>8.8220000000000007E-2</v>
+      </c>
+      <c r="C13" s="53">
+        <v>0.1658</v>
+      </c>
+      <c r="D13" s="53">
+        <v>0.53200000000000003</v>
+      </c>
+      <c r="E13" s="55">
+        <v>0.59467700000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="53">
+        <v>0.12934000000000001</v>
+      </c>
+      <c r="C14" s="53">
+        <v>0.15945000000000001</v>
+      </c>
+      <c r="D14" s="53">
+        <v>0.81100000000000005</v>
+      </c>
+      <c r="E14" s="55">
+        <v>0.41727700000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="53">
+        <v>-0.15859999999999999</v>
+      </c>
+      <c r="C15" s="53">
+        <v>0.19</v>
+      </c>
+      <c r="D15" s="53">
+        <v>-0.83499999999999996</v>
+      </c>
+      <c r="E15" s="55">
+        <v>0.403866</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="53">
+        <v>-2.2200000000000001E-2</v>
+      </c>
+      <c r="C16" s="53">
+        <v>0.20202999999999999</v>
+      </c>
+      <c r="D16" s="53">
+        <v>-0.11</v>
+      </c>
+      <c r="E16" s="55">
+        <v>0.91251599999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="56" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="66">
+        <v>-0.56679000000000002</v>
+      </c>
+      <c r="C17" s="66">
+        <v>0.19993</v>
+      </c>
+      <c r="D17" s="66">
+        <v>-2.835</v>
+      </c>
+      <c r="E17" s="67">
+        <v>4.5830000000000003E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="13" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE359B3F-A0ED-4E0B-ADAE-ED9507B865F0}">
+  <dimension ref="A1:Q31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="3" max="3" width="8.21875" customWidth="1"/>
+    <col min="4" max="4" width="1.44140625" customWidth="1"/>
+    <col min="5" max="5" width="27.88671875" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" customWidth="1"/>
+    <col min="13" max="13" width="17.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="28">
+        <v>1998.34</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="53">
+        <v>0.35139999999999999</v>
+      </c>
+      <c r="G4" s="53">
+        <v>0.1439</v>
+      </c>
+      <c r="H4" s="54">
+        <v>2.4420000000000002</v>
+      </c>
+      <c r="I4" s="64">
+        <v>1.46E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="28">
+        <v>372.49</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="53">
+        <v>1.5983000000000001</v>
+      </c>
+      <c r="G5" s="53">
+        <v>0.12759999999999999</v>
+      </c>
+      <c r="H5" s="54">
+        <v>12.523999999999999</v>
+      </c>
+      <c r="I5" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="27">
+        <v>2.36</v>
+      </c>
+      <c r="C6" s="62">
+        <v>0.124</v>
+      </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="53">
+        <v>-2.0356000000000001</v>
+      </c>
+      <c r="G6" s="53">
+        <v>0.18559999999999999</v>
+      </c>
+      <c r="H6" s="54">
+        <v>-10.968999999999999</v>
+      </c>
+      <c r="I6" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q6" s="1"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="28">
+        <v>9.76</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" s="53">
+        <v>-1.0350999999999999</v>
+      </c>
+      <c r="G7" s="53">
+        <v>0.15790000000000001</v>
+      </c>
+      <c r="H7" s="54">
+        <v>-6.5540000000000003</v>
+      </c>
+      <c r="I7" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="27">
+        <v>0.6</v>
+      </c>
+      <c r="C8" s="62">
+        <v>0.438</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" s="53">
+        <v>-0.55400000000000005</v>
+      </c>
+      <c r="G8" s="53">
+        <v>0.26140000000000002</v>
+      </c>
+      <c r="H8" s="62">
+        <v>-2.12</v>
+      </c>
+      <c r="I8" s="33">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="P8" s="1"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="27">
+        <v>0.8</v>
+      </c>
+      <c r="C9" s="55">
+        <v>0.85</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="32"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="28">
+        <v>10.74</v>
+      </c>
+      <c r="C10" s="33">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="32"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="H11" s="18"/>
+      <c r="I11" s="19"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="11">
+        <v>4111</v>
+      </c>
+      <c r="C12" s="31">
+        <v>4227</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0.38600000000000001</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0.62</v>
+      </c>
+      <c r="H12" s="14"/>
+      <c r="I12" s="20"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11">
+        <v>4686</v>
+      </c>
+      <c r="C13" s="22"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" s="14">
+        <v>0.02</v>
+      </c>
+      <c r="H13" s="14"/>
+      <c r="I13" s="20"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6">
+        <v>42</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="6"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="12">
+        <v>2</v>
+      </c>
+      <c r="C15" s="24"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="12"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="39"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="33">
+        <v>2231.06</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" s="53">
+        <v>0.29870000000000002</v>
+      </c>
+      <c r="G19" s="53">
+        <v>0.65169999999999995</v>
+      </c>
+      <c r="H19" s="53">
+        <v>0.45800000000000002</v>
+      </c>
+      <c r="I19" s="62">
+        <v>0.64671199999999995</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="33">
+        <v>136.72999999999999</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="53">
+        <v>1.7978000000000001</v>
+      </c>
+      <c r="G20" s="53">
+        <v>0.13350000000000001</v>
+      </c>
+      <c r="H20" s="53">
+        <v>13.471</v>
+      </c>
+      <c r="I20" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="33">
+        <v>6.58</v>
+      </c>
+      <c r="C21" s="64">
+        <v>0.01</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="53">
+        <v>-1.3940999999999999</v>
+      </c>
+      <c r="G21" s="53">
+        <v>0.1658</v>
+      </c>
+      <c r="H21" s="53">
+        <v>-8.407</v>
+      </c>
+      <c r="I21" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="33">
+        <v>83.62</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="53">
+        <v>-1.1083000000000001</v>
+      </c>
+      <c r="G22" s="53">
+        <v>0.17430000000000001</v>
+      </c>
+      <c r="H22" s="53">
+        <v>-6.3579999999999997</v>
+      </c>
+      <c r="I22" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q22" s="1"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="62">
+        <v>2.67</v>
+      </c>
+      <c r="C23" s="62">
+        <v>0.10199999999999999</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F23" s="53">
+        <v>-0.6663</v>
+      </c>
+      <c r="G23" s="53">
+        <v>0.17799999999999999</v>
+      </c>
+      <c r="H23" s="53">
+        <v>-3.7429999999999999</v>
+      </c>
+      <c r="I23" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q23" s="1"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="62">
+        <v>1.28</v>
+      </c>
+      <c r="C24" s="62">
+        <v>0.73299999999999998</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="53">
+        <v>-0.36890000000000001</v>
+      </c>
+      <c r="G24" s="53">
+        <v>0.16089999999999999</v>
+      </c>
+      <c r="H24" s="53">
+        <v>-2.2930000000000001</v>
+      </c>
+      <c r="I24" s="64">
+        <v>2.1864999999999999E-2</v>
+      </c>
+      <c r="Q24" s="1"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="62">
+        <v>3.71</v>
+      </c>
+      <c r="C25" s="62">
+        <v>0.29499999999999998</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F25" s="53">
+        <v>0.64770000000000005</v>
+      </c>
+      <c r="G25" s="53">
+        <v>0.21210000000000001</v>
+      </c>
+      <c r="H25" s="53">
+        <v>3.0539999999999998</v>
+      </c>
+      <c r="I25" s="64">
+        <v>2.2599999999999999E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C26" s="25"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F26" s="53">
+        <v>1.2291000000000001</v>
+      </c>
+      <c r="G26" s="53">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="H26" s="53">
+        <v>5.0789999999999997</v>
+      </c>
+      <c r="I26" s="35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="9"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="H27" s="18"/>
+      <c r="I27" s="19"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="11">
+        <v>3688</v>
+      </c>
+      <c r="C28" s="31">
+        <v>3804</v>
+      </c>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" s="14">
+        <v>0.76490000000000002</v>
+      </c>
+      <c r="G28" s="14">
+        <v>0.87460000000000004</v>
+      </c>
+      <c r="H28" s="14"/>
+      <c r="I28" s="20"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="11">
+        <v>4685</v>
+      </c>
+      <c r="C29" s="22"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" s="14">
+        <v>0.78810000000000002</v>
+      </c>
+      <c r="G29" s="14">
+        <v>0.88770000000000004</v>
+      </c>
+      <c r="H29" s="14"/>
+      <c r="I29" s="20"/>
+      <c r="Q29" s="1"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="6">
+        <v>42</v>
+      </c>
+      <c r="C30" s="22"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="6"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="12">
+        <v>2</v>
+      </c>
+      <c r="C31" s="24"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="B17:I17"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>